<commit_message>
Add README, finalise repo for GitHub publication
- Comprehensive English README with abstract, headline results,
  embedded figures, methodology explanation, repo layout, and
  reproduction instructions.
- .gitignore extended to exclude raw API caches (V2/data/raw/),
  copyrighted Literature PDFs, personal Submission PDF, LaTeX
  build artefacts, and obsolete PROJECT_CONTEXT snapshots.
- Removes deleted scratch files (audio_script, explanation.mp3,
  old context copies) from index.
- Adds remaining phase scripts (phase0, phase0b, phase10-12),
  generate_figures.py, and all phase output CSVs / figures.
</commit_message>
<xml_diff>
--- a/V2/BESS SA.xlsx
+++ b/V2/BESS SA.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10208"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/webshape/Library/Mobile Documents/com~apple~CloudDocs/Dateien/UCL/Econometrics/Assessment/V2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4661C4EC-0DED-3245-A245-D22B24CC956B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62B9EE8A-C690-BA40-9FE3-99663F90D8EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="5640" yWindow="4960" windowWidth="28040" windowHeight="17440" xr2:uid="{F9359397-F4F1-D047-8483-3AD39FC29116}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="26">
   <si>
     <t>Name der Anlage</t>
   </si>
@@ -60,12 +60,6 @@
   </si>
   <si>
     <t>Christies Beach</t>
-  </si>
-  <si>
-    <t>Happy Valley</t>
-  </si>
-  <si>
-    <t>Bolivar</t>
   </si>
   <si>
     <t>Adelaide Desalination</t>
@@ -249,8 +243,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{CA33EF9C-7BC5-D843-8BE7-A99C26FD7FEF}" name="Table1" displayName="Table1" ref="A1:F13" totalsRowShown="0" headerRowDxfId="3">
-  <autoFilter ref="A1:F13" xr:uid="{CA33EF9C-7BC5-D843-8BE7-A99C26FD7FEF}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{CA33EF9C-7BC5-D843-8BE7-A99C26FD7FEF}" name="Table1" displayName="Table1" ref="A1:F11" totalsRowShown="0" headerRowDxfId="3">
+  <autoFilter ref="A1:F11" xr:uid="{CA33EF9C-7BC5-D843-8BE7-A99C26FD7FEF}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{2763A2BA-F120-9A4C-9D9F-4F4489345B83}" name="Name der Anlage" dataDxfId="2"/>
     <tableColumn id="2" xr3:uid="{35573FAE-CBA3-4348-978E-3C52F1E9D04C}" name="freigegebene Leistung (MW)"/>
@@ -580,7 +574,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DCA82F0D-5F41-D543-AD03-6B163F69116A}">
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="38" customWidth="1"/>
@@ -595,7 +589,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="C1" s="4" t="s">
         <v>1</v>
@@ -604,10 +598,10 @@
         <v>2</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
@@ -625,7 +619,7 @@
       </c>
       <c r="E2" s="2"/>
       <c r="F2" s="3" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
@@ -643,7 +637,7 @@
       </c>
       <c r="E3" s="2"/>
       <c r="F3" s="3" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="G3">
         <v>200</v>
@@ -667,7 +661,7 @@
       </c>
       <c r="E4" s="2"/>
       <c r="F4" s="3" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.2">
@@ -685,7 +679,7 @@
       </c>
       <c r="E5" s="2"/>
       <c r="F5" s="3" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
@@ -702,10 +696,10 @@
         <v>44621</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="F6" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
@@ -713,16 +707,19 @@
         <v>8</v>
       </c>
       <c r="B7">
-        <v>4</v>
+        <v>6.2</v>
       </c>
       <c r="C7">
-        <v>8.8000000000000007</v>
+        <v>13</v>
       </c>
       <c r="D7" s="2">
-        <v>44713</v>
+        <v>44317</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>27</v>
+        <v>25</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.2">
@@ -730,16 +727,17 @@
         <v>9</v>
       </c>
       <c r="B8">
-        <v>2</v>
+        <v>25</v>
       </c>
       <c r="C8">
-        <v>5</v>
+        <v>52</v>
       </c>
       <c r="D8" s="2">
-        <v>44593</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>27</v>
+        <v>43800</v>
+      </c>
+      <c r="E8" s="2"/>
+      <c r="F8" s="3" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
@@ -747,19 +745,17 @@
         <v>10</v>
       </c>
       <c r="B9">
-        <v>6.2</v>
+        <v>30</v>
       </c>
       <c r="C9">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D9" s="2">
-        <v>44317</v>
-      </c>
-      <c r="E9" s="2" t="s">
-        <v>27</v>
-      </c>
+        <v>43435</v>
+      </c>
+      <c r="E9" s="2"/>
       <c r="F9" s="3" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.2">
@@ -767,80 +763,44 @@
         <v>11</v>
       </c>
       <c r="B10">
-        <v>25</v>
+        <v>100</v>
       </c>
       <c r="C10">
-        <v>52</v>
+        <v>129</v>
       </c>
       <c r="D10" s="2">
-        <v>43800</v>
+        <v>43009</v>
       </c>
       <c r="E10" s="2"/>
       <c r="F10" s="3" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="B11">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="C11">
-        <v>8</v>
+        <v>64.5</v>
       </c>
       <c r="D11" s="2">
-        <v>43435</v>
+        <v>44075</v>
       </c>
       <c r="E11" s="2"/>
       <c r="F11" s="3" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A12" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B12">
-        <v>100</v>
-      </c>
-      <c r="C12">
-        <v>129</v>
-      </c>
-      <c r="D12" s="2">
-        <v>43009</v>
-      </c>
-      <c r="E12" s="2"/>
-      <c r="F12" s="3" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A13" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="B13">
-        <v>50</v>
-      </c>
-      <c r="C13">
-        <v>64.5</v>
-      </c>
-      <c r="D13" s="2">
-        <v>44075</v>
-      </c>
-      <c r="E13" s="2"/>
-      <c r="F13" s="3" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="F12" r:id="rId1" xr:uid="{4CEB9EFB-3909-734F-8D5B-2D62C16B57F1}"/>
-    <hyperlink ref="F13" r:id="rId2" xr:uid="{5CBD9CDA-9F10-2543-BB83-7F380535AAD3}"/>
-    <hyperlink ref="F11" r:id="rId3" xr:uid="{E57A5F65-730B-8944-ACA5-46C9BAC40736}"/>
-    <hyperlink ref="F10" r:id="rId4" xr:uid="{B997338D-5070-F64F-B553-342B499A0800}"/>
-    <hyperlink ref="F9" r:id="rId5" xr:uid="{6EDEDE20-0E07-DB41-AD93-D89A8199BE43}"/>
+    <hyperlink ref="F10" r:id="rId1" xr:uid="{4CEB9EFB-3909-734F-8D5B-2D62C16B57F1}"/>
+    <hyperlink ref="F11" r:id="rId2" xr:uid="{5CBD9CDA-9F10-2543-BB83-7F380535AAD3}"/>
+    <hyperlink ref="F9" r:id="rId3" xr:uid="{E57A5F65-730B-8944-ACA5-46C9BAC40736}"/>
+    <hyperlink ref="F8" r:id="rId4" xr:uid="{B997338D-5070-F64F-B553-342B499A0800}"/>
+    <hyperlink ref="F7" r:id="rId5" xr:uid="{6EDEDE20-0E07-DB41-AD93-D89A8199BE43}"/>
     <hyperlink ref="F2" r:id="rId6" xr:uid="{8D5F46AA-618A-0847-ACF9-BD8D7DE41403}"/>
     <hyperlink ref="F3" r:id="rId7" xr:uid="{4844DFDA-1186-5948-9671-ED1FB313E60C}"/>
     <hyperlink ref="F4" r:id="rId8" xr:uid="{E6207573-9B01-234D-9131-05A576B749B0}"/>

</xml_diff>